<commit_message>
feat: ampliar planes, historiales y ofertas hasta el bloque 6
</commit_message>
<xml_diff>
--- a/Parte 1/data/CEmestre_datos.xlsx
+++ b/Parte 1/data/CEmestre_datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josaq\Downloads\CEmestre\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josaq\Downloads\Proyecto---Paradigmas-de-Programaci-n\Parte 1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B99B30-B03A-4760-96BF-04751FDF3C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BBA47A-4812-4ACA-BEDF-29771235317E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5873" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6571" uniqueCount="511">
   <si>
     <t>codigo_plan</t>
   </si>
@@ -1311,13 +1311,262 @@
   </si>
   <si>
     <t>CFH (FH1000): por indicación del profesor se modela como un solo curso con un horario representativo, en este caso: FH0035 Globalización y humanismo, MAR 17:00-19:50</t>
+  </si>
+  <si>
+    <t>CE1107</t>
+  </si>
+  <si>
+    <t>Fundamentos de arquitectura de computadores</t>
+  </si>
+  <si>
+    <t>CE3101</t>
+  </si>
+  <si>
+    <t>Bases de datos</t>
+  </si>
+  <si>
+    <t>CE3201</t>
+  </si>
+  <si>
+    <t>Taller de diseño digital</t>
+  </si>
+  <si>
+    <t>MA2105</t>
+  </si>
+  <si>
+    <t>Ecuaciones diferenciales</t>
+  </si>
+  <si>
+    <t>PI5516</t>
+  </si>
+  <si>
+    <t>Ingeniería económica</t>
+  </si>
+  <si>
+    <t>CE1108</t>
+  </si>
+  <si>
+    <t>Compiladores e intérpretes</t>
+  </si>
+  <si>
+    <t>CE4301</t>
+  </si>
+  <si>
+    <t>CE1109</t>
+  </si>
+  <si>
+    <t>Circuitos analógicos</t>
+  </si>
+  <si>
+    <t>EL2207,SO4604</t>
+  </si>
+  <si>
+    <t>CE1110</t>
+  </si>
+  <si>
+    <t>Análisis de señales mixtas</t>
+  </si>
+  <si>
+    <t>EL2114,MA2105</t>
+  </si>
+  <si>
+    <t>Arquitectura de computadores I</t>
+  </si>
+  <si>
+    <t>CE1107,CE3201</t>
+  </si>
+  <si>
+    <t>CI3203</t>
+  </si>
+  <si>
+    <t>Inglés especializado para ingenierías en computadores</t>
+  </si>
+  <si>
+    <t>CS3404</t>
+  </si>
+  <si>
+    <t>Seminario de ética para la ingeniería</t>
+  </si>
+  <si>
+    <t>MI3138</t>
+  </si>
+  <si>
+    <t>Máquinas y equipos</t>
+  </si>
+  <si>
+    <t>PI3308</t>
+  </si>
+  <si>
+    <t>Estudio del trabajo II</t>
+  </si>
+  <si>
+    <t>PI3407</t>
+  </si>
+  <si>
+    <t>Computación industrial</t>
+  </si>
+  <si>
+    <t>CA2125,CI1231</t>
+  </si>
+  <si>
+    <t>PI3612</t>
+  </si>
+  <si>
+    <t>Probabilidad y estadística II</t>
+  </si>
+  <si>
+    <t>MA1103,PI2610</t>
+  </si>
+  <si>
+    <t>CM3207</t>
+  </si>
+  <si>
+    <t>Métodos numéricos para ingeniería</t>
+  </si>
+  <si>
+    <t>MA2105,PI3407</t>
+  </si>
+  <si>
+    <t>ME2208</t>
+  </si>
+  <si>
+    <t>Ciencias de los materiales</t>
+  </si>
+  <si>
+    <t>FI1102,QU1107</t>
+  </si>
+  <si>
+    <t>PI3206</t>
+  </si>
+  <si>
+    <t>Logística y administración de la cadena de abastecimiento</t>
+  </si>
+  <si>
+    <t>PI3603</t>
+  </si>
+  <si>
+    <t>PI3403</t>
+  </si>
+  <si>
+    <t>Sistema de información</t>
+  </si>
+  <si>
+    <t>PI3512</t>
+  </si>
+  <si>
+    <t>Dirección de personal</t>
+  </si>
+  <si>
+    <t>CS2303,PI3308</t>
+  </si>
+  <si>
+    <t>Investigación de operaciones I</t>
+  </si>
+  <si>
+    <t>CHAVARRIA ZAMORA LUIS</t>
+  </si>
+  <si>
+    <t>CALDERON PRADO KIMBERLY</t>
+  </si>
+  <si>
+    <t>08:30</t>
+  </si>
+  <si>
+    <t>BRENES GOMEZ RANDALL</t>
+  </si>
+  <si>
+    <t>MARIN SANCHEZ MARIO</t>
+  </si>
+  <si>
+    <t>CHACON ROJAS FERNANDO</t>
+  </si>
+  <si>
+    <t>FARAH GUZMAN BILJHANA SHAKIRA</t>
+  </si>
+  <si>
+    <t>LEITON JIMENEZ JASON</t>
+  </si>
+  <si>
+    <t>ARAYA RODRIGUEZ LISANDRO</t>
+  </si>
+  <si>
+    <t>GONZALEZ GOMEZ JEFERSON</t>
+  </si>
+  <si>
+    <t>JIMENEZ RODRIGUEZ ROXANA</t>
+  </si>
+  <si>
+    <t>VARGAS ELIZONDO CELSO</t>
+  </si>
+  <si>
+    <t>GUZMAN CONEJO JOSHUA</t>
+  </si>
+  <si>
+    <t>LEMAITRE GONZALEZ ESTEBAN</t>
+  </si>
+  <si>
+    <t>SALAS CERDAS LISS</t>
+  </si>
+  <si>
+    <t>MONGE RUIZ OSCAR EDUARDO</t>
+  </si>
+  <si>
+    <t>HASBUM FERNANDEZ IVANNIA</t>
+  </si>
+  <si>
+    <t>BRENES NAVARRO BALAM</t>
+  </si>
+  <si>
+    <t>CASASOLA RIVERA WILMER</t>
+  </si>
+  <si>
+    <t>PRENDAS SOLANO JORGE</t>
+  </si>
+  <si>
+    <t>CEDEÑO CAMACHO MAURICIO</t>
+  </si>
+  <si>
+    <t>CHINE POLITO BRUNO</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ QUESADA LARIA FABIOLA</t>
+  </si>
+  <si>
+    <t>CAVERO QUESADA ANDREA</t>
+  </si>
+  <si>
+    <t>VEGA GARITA VICTOR</t>
+  </si>
+  <si>
+    <t>SANCHEZ CORDERO CARLOS ALBERTO</t>
+  </si>
+  <si>
+    <t>ARIAS RAMIREZ DENNIS</t>
+  </si>
+  <si>
+    <t>VARGAS GOMEZ PABLO JOSE</t>
+  </si>
+  <si>
+    <t>STRADI GRANADOS BENITO</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ ROJAS ALFREDO</t>
+  </si>
+  <si>
+    <t>ARAYA MENESES IVAN</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ MENDEZ FRANCISCO</t>
+  </si>
+  <si>
+    <t>CALDERON ARCE CINDY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1329,21 +1578,50 @@
       <b/>
       <sz val="12"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF808080"/>
+      <name val="Helvetica"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1376,7 +1654,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1384,6 +1662,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1808,7 +2091,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2456,7 +2739,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="7" t="s">
         <v>123</v>
       </c>
       <c r="B28" s="5" t="s">
@@ -2530,7 +2813,7 @@
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="7" t="s">
         <v>129</v>
       </c>
       <c r="B31" s="5" t="s">
@@ -2550,6 +2833,248 @@
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="C32" s="8">
+        <v>4</v>
+      </c>
+      <c r="D32" s="8">
+        <v>12</v>
+      </c>
+      <c r="E32" s="9">
+        <v>5</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="C33" s="9">
+        <v>4</v>
+      </c>
+      <c r="D33" s="9">
+        <v>12</v>
+      </c>
+      <c r="E33" s="9">
+        <v>5</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C34" s="9">
+        <v>2</v>
+      </c>
+      <c r="D34" s="9">
+        <v>6</v>
+      </c>
+      <c r="E34" s="9">
+        <v>5</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="C35" s="9">
+        <v>4</v>
+      </c>
+      <c r="D35" s="9">
+        <v>4</v>
+      </c>
+      <c r="E35" s="9">
+        <v>5</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="C36" s="9">
+        <v>3</v>
+      </c>
+      <c r="D36" s="9">
+        <v>4</v>
+      </c>
+      <c r="E36" s="9">
+        <v>5</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="C37" s="9">
+        <v>4</v>
+      </c>
+      <c r="D37" s="9">
+        <v>12</v>
+      </c>
+      <c r="E37" s="9">
+        <v>6</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="C38" s="9">
+        <v>4</v>
+      </c>
+      <c r="D38" s="9">
+        <v>12</v>
+      </c>
+      <c r="E38" s="9">
+        <v>6</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="C39" s="9">
+        <v>4</v>
+      </c>
+      <c r="D39" s="9">
+        <v>12</v>
+      </c>
+      <c r="E39" s="9">
+        <v>6</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="C40" s="9">
+        <v>4</v>
+      </c>
+      <c r="D40" s="9">
+        <v>12</v>
+      </c>
+      <c r="E40" s="9">
+        <v>6</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="C41" s="9">
+        <v>2</v>
+      </c>
+      <c r="D41" s="9">
+        <v>6</v>
+      </c>
+      <c r="E41" s="9">
+        <v>6</v>
+      </c>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2560,7 +3085,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3014,7 +3539,7 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="7" t="s">
         <v>148</v>
       </c>
       <c r="B20" s="5" t="s">
@@ -3330,7 +3855,7 @@
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="7" t="s">
         <v>166</v>
       </c>
       <c r="B33" s="5" t="s">
@@ -3350,6 +3875,296 @@
       </c>
       <c r="G33" s="5"/>
       <c r="H33" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C34" s="9">
+        <v>2</v>
+      </c>
+      <c r="D34" s="9">
+        <v>5</v>
+      </c>
+      <c r="E34" s="9">
+        <v>5</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="C35" s="9">
+        <v>4</v>
+      </c>
+      <c r="D35" s="9">
+        <v>4</v>
+      </c>
+      <c r="E35" s="9">
+        <v>5</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="C36" s="9">
+        <v>3</v>
+      </c>
+      <c r="D36" s="9">
+        <v>4</v>
+      </c>
+      <c r="E36" s="9">
+        <v>5</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="C37" s="9">
+        <v>3</v>
+      </c>
+      <c r="D37" s="9">
+        <v>4</v>
+      </c>
+      <c r="E37" s="9">
+        <v>5</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C38" s="9">
+        <v>3</v>
+      </c>
+      <c r="D38" s="9">
+        <v>3</v>
+      </c>
+      <c r="E38" s="9">
+        <v>5</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="C39" s="9">
+        <v>3</v>
+      </c>
+      <c r="D39" s="9">
+        <v>9</v>
+      </c>
+      <c r="E39" s="9">
+        <v>5</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C40" s="9">
+        <v>3</v>
+      </c>
+      <c r="D40" s="9">
+        <v>4</v>
+      </c>
+      <c r="E40" s="9">
+        <v>6</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="C41" s="9">
+        <v>3</v>
+      </c>
+      <c r="D41" s="9">
+        <v>3</v>
+      </c>
+      <c r="E41" s="9">
+        <v>6</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="C42" s="9">
+        <v>3</v>
+      </c>
+      <c r="D42" s="9">
+        <v>3</v>
+      </c>
+      <c r="E42" s="9">
+        <v>6</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="C43" s="9">
+        <v>3</v>
+      </c>
+      <c r="D43" s="9">
+        <v>3</v>
+      </c>
+      <c r="E43" s="9">
+        <v>6</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="C44" s="9">
+        <v>3</v>
+      </c>
+      <c r="D44" s="9">
+        <v>4</v>
+      </c>
+      <c r="E44" s="9">
+        <v>6</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="C45" s="9">
+        <v>3</v>
+      </c>
+      <c r="D45" s="9">
+        <v>4</v>
+      </c>
+      <c r="E45" s="9">
+        <v>6</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5" t="s">
         <v>71</v>
       </c>
     </row>
@@ -3360,7 +4175,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="11" customWidth="1"/>
@@ -3651,9 +4466,99 @@
       </c>
       <c r="C31" s="6"/>
     </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C32" s="6"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C33" s="6"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C34" s="6"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C36" s="6"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C37" s="6"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="6"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C40" s="6"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C41" s="6"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Solo SI o NO" sqref="B2:B31" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Solo SI o NO" sqref="B2:B41" xr:uid="{8DF65921-83EC-468C-A9FE-FCCE254BD701}">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3663,7 +4568,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="11" customWidth="1"/>
@@ -3970,9 +4875,117 @@
       </c>
       <c r="C33" s="6"/>
     </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C34" s="6"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C35" s="6"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C36" s="6"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C37" s="6"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C38" s="6"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="6"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C40" s="6"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C41" s="6"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C42" s="6"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C43" s="6"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C44" s="6"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C45" s="6"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Solo SI o NO" sqref="B2:B33" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Solo SI o NO" sqref="B2:B45" xr:uid="{1F960768-9DDB-4F00-AB98-88DBEAA24558}">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3982,7 +4995,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G382"/>
+  <dimension ref="A1:G421"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -12779,6 +13792,903 @@
         <v>346</v>
       </c>
     </row>
+    <row r="383" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A383" t="s">
+        <v>428</v>
+      </c>
+      <c r="B383">
+        <v>1</v>
+      </c>
+      <c r="C383" t="s">
+        <v>184</v>
+      </c>
+      <c r="D383" t="s">
+        <v>185</v>
+      </c>
+      <c r="E383" t="s">
+        <v>186</v>
+      </c>
+      <c r="F383" t="s">
+        <v>182</v>
+      </c>
+      <c r="G383" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="384" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A384" t="s">
+        <v>428</v>
+      </c>
+      <c r="B384">
+        <v>1</v>
+      </c>
+      <c r="C384" t="s">
+        <v>179</v>
+      </c>
+      <c r="D384" t="s">
+        <v>185</v>
+      </c>
+      <c r="E384" t="s">
+        <v>186</v>
+      </c>
+      <c r="F384" t="s">
+        <v>182</v>
+      </c>
+      <c r="G384" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="385" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A385" t="s">
+        <v>430</v>
+      </c>
+      <c r="B385">
+        <v>2</v>
+      </c>
+      <c r="C385" t="s">
+        <v>187</v>
+      </c>
+      <c r="D385" t="s">
+        <v>200</v>
+      </c>
+      <c r="E385" t="s">
+        <v>201</v>
+      </c>
+      <c r="F385" t="s">
+        <v>182</v>
+      </c>
+      <c r="G385" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="386" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>430</v>
+      </c>
+      <c r="B386">
+        <v>2</v>
+      </c>
+      <c r="C386" t="s">
+        <v>191</v>
+      </c>
+      <c r="D386" t="s">
+        <v>200</v>
+      </c>
+      <c r="E386" t="s">
+        <v>201</v>
+      </c>
+      <c r="F386" t="s">
+        <v>182</v>
+      </c>
+      <c r="G386" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="387" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>430</v>
+      </c>
+      <c r="B387">
+        <v>1</v>
+      </c>
+      <c r="C387" t="s">
+        <v>187</v>
+      </c>
+      <c r="D387" t="s">
+        <v>200</v>
+      </c>
+      <c r="E387" t="s">
+        <v>201</v>
+      </c>
+      <c r="F387" t="s">
+        <v>182</v>
+      </c>
+      <c r="G387" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="388" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>430</v>
+      </c>
+      <c r="B388">
+        <v>1</v>
+      </c>
+      <c r="C388" t="s">
+        <v>191</v>
+      </c>
+      <c r="D388" t="s">
+        <v>200</v>
+      </c>
+      <c r="E388" t="s">
+        <v>201</v>
+      </c>
+      <c r="F388" t="s">
+        <v>182</v>
+      </c>
+      <c r="G388" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="389" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>432</v>
+      </c>
+      <c r="B389">
+        <v>1</v>
+      </c>
+      <c r="C389" t="s">
+        <v>184</v>
+      </c>
+      <c r="D389" t="s">
+        <v>208</v>
+      </c>
+      <c r="E389" t="s">
+        <v>239</v>
+      </c>
+      <c r="F389" t="s">
+        <v>182</v>
+      </c>
+      <c r="G389" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="390" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>432</v>
+      </c>
+      <c r="B390">
+        <v>1</v>
+      </c>
+      <c r="C390" t="s">
+        <v>275</v>
+      </c>
+      <c r="D390" t="s">
+        <v>480</v>
+      </c>
+      <c r="E390" t="s">
+        <v>212</v>
+      </c>
+      <c r="F390" t="s">
+        <v>182</v>
+      </c>
+      <c r="G390" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="391" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>432</v>
+      </c>
+      <c r="B391">
+        <v>2</v>
+      </c>
+      <c r="C391" t="s">
+        <v>179</v>
+      </c>
+      <c r="D391" t="s">
+        <v>208</v>
+      </c>
+      <c r="E391" t="s">
+        <v>239</v>
+      </c>
+      <c r="F391" t="s">
+        <v>289</v>
+      </c>
+      <c r="G391" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="392" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>432</v>
+      </c>
+      <c r="B392">
+        <v>2</v>
+      </c>
+      <c r="C392" t="s">
+        <v>275</v>
+      </c>
+      <c r="D392" t="s">
+        <v>279</v>
+      </c>
+      <c r="E392" t="s">
+        <v>206</v>
+      </c>
+      <c r="F392" t="s">
+        <v>289</v>
+      </c>
+      <c r="G392" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="393" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>434</v>
+      </c>
+      <c r="B393">
+        <v>5</v>
+      </c>
+      <c r="C393" t="s">
+        <v>275</v>
+      </c>
+      <c r="D393" t="s">
+        <v>180</v>
+      </c>
+      <c r="E393" t="s">
+        <v>186</v>
+      </c>
+      <c r="F393" t="s">
+        <v>247</v>
+      </c>
+      <c r="G393" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="394" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
+        <v>434</v>
+      </c>
+      <c r="B394">
+        <v>1</v>
+      </c>
+      <c r="C394" t="s">
+        <v>184</v>
+      </c>
+      <c r="D394" t="s">
+        <v>180</v>
+      </c>
+      <c r="E394" t="s">
+        <v>181</v>
+      </c>
+      <c r="F394" t="s">
+        <v>196</v>
+      </c>
+      <c r="G394" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A395" t="s">
+        <v>434</v>
+      </c>
+      <c r="B395">
+        <v>1</v>
+      </c>
+      <c r="C395" t="s">
+        <v>179</v>
+      </c>
+      <c r="D395" t="s">
+        <v>180</v>
+      </c>
+      <c r="E395" t="s">
+        <v>181</v>
+      </c>
+      <c r="F395" t="s">
+        <v>196</v>
+      </c>
+      <c r="G395" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="396" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>434</v>
+      </c>
+      <c r="B396">
+        <v>3</v>
+      </c>
+      <c r="C396" t="s">
+        <v>184</v>
+      </c>
+      <c r="D396" t="s">
+        <v>185</v>
+      </c>
+      <c r="E396" t="s">
+        <v>186</v>
+      </c>
+      <c r="F396" t="s">
+        <v>196</v>
+      </c>
+      <c r="G396" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="397" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>434</v>
+      </c>
+      <c r="B397">
+        <v>3</v>
+      </c>
+      <c r="C397" t="s">
+        <v>179</v>
+      </c>
+      <c r="D397" t="s">
+        <v>185</v>
+      </c>
+      <c r="E397" t="s">
+        <v>186</v>
+      </c>
+      <c r="F397" t="s">
+        <v>196</v>
+      </c>
+      <c r="G397" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="398" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A398" t="s">
+        <v>434</v>
+      </c>
+      <c r="B398">
+        <v>2</v>
+      </c>
+      <c r="C398" t="s">
+        <v>187</v>
+      </c>
+      <c r="D398" t="s">
+        <v>208</v>
+      </c>
+      <c r="E398" t="s">
+        <v>239</v>
+      </c>
+      <c r="F398" t="s">
+        <v>196</v>
+      </c>
+      <c r="G398" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="399" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A399" t="s">
+        <v>434</v>
+      </c>
+      <c r="B399">
+        <v>2</v>
+      </c>
+      <c r="C399" t="s">
+        <v>191</v>
+      </c>
+      <c r="D399" t="s">
+        <v>208</v>
+      </c>
+      <c r="E399" t="s">
+        <v>239</v>
+      </c>
+      <c r="F399" t="s">
+        <v>196</v>
+      </c>
+      <c r="G399" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="400" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A400" t="s">
+        <v>434</v>
+      </c>
+      <c r="B400">
+        <v>4</v>
+      </c>
+      <c r="C400" t="s">
+        <v>187</v>
+      </c>
+      <c r="D400" t="s">
+        <v>188</v>
+      </c>
+      <c r="E400" t="s">
+        <v>189</v>
+      </c>
+      <c r="F400" t="s">
+        <v>182</v>
+      </c>
+      <c r="G400" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="401" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A401" t="s">
+        <v>434</v>
+      </c>
+      <c r="B401">
+        <v>4</v>
+      </c>
+      <c r="C401" t="s">
+        <v>191</v>
+      </c>
+      <c r="D401" t="s">
+        <v>188</v>
+      </c>
+      <c r="E401" t="s">
+        <v>189</v>
+      </c>
+      <c r="F401" t="s">
+        <v>182</v>
+      </c>
+      <c r="G401" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="402" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>434</v>
+      </c>
+      <c r="B402">
+        <v>8</v>
+      </c>
+      <c r="C402" t="s">
+        <v>184</v>
+      </c>
+      <c r="D402" t="s">
+        <v>188</v>
+      </c>
+      <c r="E402" t="s">
+        <v>189</v>
+      </c>
+      <c r="F402" t="s">
+        <v>289</v>
+      </c>
+      <c r="G402" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="403" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>434</v>
+      </c>
+      <c r="B403">
+        <v>8</v>
+      </c>
+      <c r="C403" t="s">
+        <v>179</v>
+      </c>
+      <c r="D403" t="s">
+        <v>188</v>
+      </c>
+      <c r="E403" t="s">
+        <v>189</v>
+      </c>
+      <c r="F403" t="s">
+        <v>289</v>
+      </c>
+      <c r="G403" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="404" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>434</v>
+      </c>
+      <c r="B404">
+        <v>9</v>
+      </c>
+      <c r="C404" t="s">
+        <v>275</v>
+      </c>
+      <c r="D404" t="s">
+        <v>180</v>
+      </c>
+      <c r="E404" t="s">
+        <v>186</v>
+      </c>
+      <c r="F404" t="s">
+        <v>247</v>
+      </c>
+      <c r="G404" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="405" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>434</v>
+      </c>
+      <c r="B405">
+        <v>6</v>
+      </c>
+      <c r="C405" t="s">
+        <v>187</v>
+      </c>
+      <c r="D405" t="s">
+        <v>192</v>
+      </c>
+      <c r="E405" t="s">
+        <v>193</v>
+      </c>
+      <c r="F405" t="s">
+        <v>196</v>
+      </c>
+      <c r="G405" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="406" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>434</v>
+      </c>
+      <c r="B406">
+        <v>6</v>
+      </c>
+      <c r="C406" t="s">
+        <v>191</v>
+      </c>
+      <c r="D406" t="s">
+        <v>192</v>
+      </c>
+      <c r="E406" t="s">
+        <v>193</v>
+      </c>
+      <c r="F406" t="s">
+        <v>196</v>
+      </c>
+      <c r="G406" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="407" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>434</v>
+      </c>
+      <c r="B407">
+        <v>10</v>
+      </c>
+      <c r="C407" t="s">
+        <v>187</v>
+      </c>
+      <c r="D407" t="s">
+        <v>185</v>
+      </c>
+      <c r="E407" t="s">
+        <v>186</v>
+      </c>
+      <c r="F407" t="s">
+        <v>196</v>
+      </c>
+      <c r="G407" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="408" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>434</v>
+      </c>
+      <c r="B408">
+        <v>10</v>
+      </c>
+      <c r="C408" t="s">
+        <v>191</v>
+      </c>
+      <c r="D408" t="s">
+        <v>185</v>
+      </c>
+      <c r="E408" t="s">
+        <v>186</v>
+      </c>
+      <c r="F408" t="s">
+        <v>196</v>
+      </c>
+      <c r="G408" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="409" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>434</v>
+      </c>
+      <c r="B409">
+        <v>7</v>
+      </c>
+      <c r="C409" t="s">
+        <v>184</v>
+      </c>
+      <c r="D409" t="s">
+        <v>188</v>
+      </c>
+      <c r="E409" t="s">
+        <v>189</v>
+      </c>
+      <c r="F409" t="s">
+        <v>196</v>
+      </c>
+      <c r="G409" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="410" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>434</v>
+      </c>
+      <c r="B410">
+        <v>7</v>
+      </c>
+      <c r="C410" t="s">
+        <v>179</v>
+      </c>
+      <c r="D410" t="s">
+        <v>188</v>
+      </c>
+      <c r="E410" t="s">
+        <v>189</v>
+      </c>
+      <c r="F410" t="s">
+        <v>196</v>
+      </c>
+      <c r="G410" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="411" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>436</v>
+      </c>
+      <c r="B411">
+        <v>1</v>
+      </c>
+      <c r="C411" t="s">
+        <v>179</v>
+      </c>
+      <c r="D411" t="s">
+        <v>188</v>
+      </c>
+      <c r="E411" t="s">
+        <v>201</v>
+      </c>
+      <c r="F411" t="s">
+        <v>196</v>
+      </c>
+      <c r="G411" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="412" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A412" t="s">
+        <v>436</v>
+      </c>
+      <c r="B412">
+        <v>2</v>
+      </c>
+      <c r="C412" t="s">
+        <v>191</v>
+      </c>
+      <c r="D412" t="s">
+        <v>188</v>
+      </c>
+      <c r="E412" t="s">
+        <v>201</v>
+      </c>
+      <c r="F412" t="s">
+        <v>216</v>
+      </c>
+      <c r="G412" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="413" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A413" t="s">
+        <v>438</v>
+      </c>
+      <c r="B413">
+        <v>1</v>
+      </c>
+      <c r="C413" t="s">
+        <v>187</v>
+      </c>
+      <c r="D413" t="s">
+        <v>208</v>
+      </c>
+      <c r="E413" t="s">
+        <v>239</v>
+      </c>
+      <c r="F413" t="s">
+        <v>182</v>
+      </c>
+      <c r="G413" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="414" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A414" t="s">
+        <v>438</v>
+      </c>
+      <c r="B414">
+        <v>1</v>
+      </c>
+      <c r="C414" t="s">
+        <v>191</v>
+      </c>
+      <c r="D414" t="s">
+        <v>208</v>
+      </c>
+      <c r="E414" t="s">
+        <v>239</v>
+      </c>
+      <c r="F414" t="s">
+        <v>182</v>
+      </c>
+      <c r="G414" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="415" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A415" t="s">
+        <v>441</v>
+      </c>
+      <c r="B415">
+        <v>1</v>
+      </c>
+      <c r="C415" t="s">
+        <v>184</v>
+      </c>
+      <c r="D415" t="s">
+        <v>188</v>
+      </c>
+      <c r="E415" t="s">
+        <v>189</v>
+      </c>
+      <c r="F415" t="s">
+        <v>182</v>
+      </c>
+      <c r="G415" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="416" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>441</v>
+      </c>
+      <c r="B416">
+        <v>1</v>
+      </c>
+      <c r="C416" t="s">
+        <v>179</v>
+      </c>
+      <c r="D416" t="s">
+        <v>188</v>
+      </c>
+      <c r="E416" t="s">
+        <v>189</v>
+      </c>
+      <c r="F416" t="s">
+        <v>182</v>
+      </c>
+      <c r="G416" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="417" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A417" t="s">
+        <v>444</v>
+      </c>
+      <c r="B417">
+        <v>1</v>
+      </c>
+      <c r="C417" t="s">
+        <v>187</v>
+      </c>
+      <c r="D417" t="s">
+        <v>185</v>
+      </c>
+      <c r="E417" t="s">
+        <v>186</v>
+      </c>
+      <c r="F417" t="s">
+        <v>182</v>
+      </c>
+      <c r="G417" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="418" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A418" t="s">
+        <v>444</v>
+      </c>
+      <c r="B418">
+        <v>1</v>
+      </c>
+      <c r="C418" t="s">
+        <v>191</v>
+      </c>
+      <c r="D418" t="s">
+        <v>185</v>
+      </c>
+      <c r="E418" t="s">
+        <v>186</v>
+      </c>
+      <c r="F418" t="s">
+        <v>182</v>
+      </c>
+      <c r="G418" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="419" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A419" t="s">
+        <v>440</v>
+      </c>
+      <c r="B419">
+        <v>1</v>
+      </c>
+      <c r="C419" t="s">
+        <v>187</v>
+      </c>
+      <c r="D419" t="s">
+        <v>192</v>
+      </c>
+      <c r="E419" t="s">
+        <v>193</v>
+      </c>
+      <c r="F419" t="s">
+        <v>182</v>
+      </c>
+      <c r="G419" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="420" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>440</v>
+      </c>
+      <c r="B420">
+        <v>1</v>
+      </c>
+      <c r="C420" t="s">
+        <v>191</v>
+      </c>
+      <c r="D420" t="s">
+        <v>192</v>
+      </c>
+      <c r="E420" t="s">
+        <v>193</v>
+      </c>
+      <c r="F420" t="s">
+        <v>182</v>
+      </c>
+      <c r="G420" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="421" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>449</v>
+      </c>
+      <c r="B421">
+        <v>1</v>
+      </c>
+      <c r="C421" t="s">
+        <v>179</v>
+      </c>
+      <c r="D421" t="s">
+        <v>208</v>
+      </c>
+      <c r="E421" t="s">
+        <v>209</v>
+      </c>
+      <c r="F421" t="s">
+        <v>196</v>
+      </c>
+      <c r="G421" t="s">
+        <v>488</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12786,7 +14696,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G506"/>
+  <dimension ref="A1:K561"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -12798,7 +14708,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="10" t="s">
         <v>61</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -24433,6 +26343,1272 @@
       </c>
       <c r="G506" s="5" t="s">
         <v>341</v>
+      </c>
+    </row>
+    <row r="507" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A507" t="s">
+        <v>451</v>
+      </c>
+      <c r="B507">
+        <v>1</v>
+      </c>
+      <c r="C507" t="s">
+        <v>179</v>
+      </c>
+      <c r="D507" t="s">
+        <v>185</v>
+      </c>
+      <c r="E507" t="s">
+        <v>206</v>
+      </c>
+      <c r="F507" t="s">
+        <v>216</v>
+      </c>
+      <c r="G507" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="508" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A508" t="s">
+        <v>434</v>
+      </c>
+      <c r="B508">
+        <v>1</v>
+      </c>
+      <c r="C508" t="s">
+        <v>184</v>
+      </c>
+      <c r="D508" t="s">
+        <v>180</v>
+      </c>
+      <c r="E508" t="s">
+        <v>181</v>
+      </c>
+      <c r="F508" t="s">
+        <v>196</v>
+      </c>
+      <c r="G508" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="509" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A509" t="s">
+        <v>434</v>
+      </c>
+      <c r="B509">
+        <v>1</v>
+      </c>
+      <c r="C509" t="s">
+        <v>179</v>
+      </c>
+      <c r="D509" t="s">
+        <v>180</v>
+      </c>
+      <c r="E509" t="s">
+        <v>181</v>
+      </c>
+      <c r="F509" t="s">
+        <v>196</v>
+      </c>
+      <c r="G509" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="510" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A510" t="s">
+        <v>453</v>
+      </c>
+      <c r="B510">
+        <v>1</v>
+      </c>
+      <c r="C510" t="s">
+        <v>204</v>
+      </c>
+      <c r="D510" t="s">
+        <v>188</v>
+      </c>
+      <c r="E510" t="s">
+        <v>201</v>
+      </c>
+      <c r="F510" t="s">
+        <v>182</v>
+      </c>
+      <c r="G510" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="511" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A511" t="s">
+        <v>455</v>
+      </c>
+      <c r="B511">
+        <v>1</v>
+      </c>
+      <c r="C511" t="s">
+        <v>179</v>
+      </c>
+      <c r="D511" t="s">
+        <v>208</v>
+      </c>
+      <c r="E511" t="s">
+        <v>193</v>
+      </c>
+      <c r="F511" t="s">
+        <v>196</v>
+      </c>
+      <c r="G511" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="512" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A512" t="s">
+        <v>457</v>
+      </c>
+      <c r="B512">
+        <v>1</v>
+      </c>
+      <c r="C512" t="s">
+        <v>184</v>
+      </c>
+      <c r="D512" t="s">
+        <v>180</v>
+      </c>
+      <c r="E512" t="s">
+        <v>212</v>
+      </c>
+      <c r="F512" t="s">
+        <v>196</v>
+      </c>
+      <c r="G512" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="513" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A513" t="s">
+        <v>460</v>
+      </c>
+      <c r="B513">
+        <v>1</v>
+      </c>
+      <c r="C513" t="s">
+        <v>204</v>
+      </c>
+      <c r="D513" t="s">
+        <v>180</v>
+      </c>
+      <c r="E513" t="s">
+        <v>186</v>
+      </c>
+      <c r="F513" t="s">
+        <v>196</v>
+      </c>
+      <c r="G513" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="514" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A514" t="s">
+        <v>451</v>
+      </c>
+      <c r="B514">
+        <v>2</v>
+      </c>
+      <c r="C514" t="s">
+        <v>204</v>
+      </c>
+      <c r="D514" t="s">
+        <v>221</v>
+      </c>
+      <c r="E514" t="s">
+        <v>201</v>
+      </c>
+      <c r="F514" t="s">
+        <v>182</v>
+      </c>
+      <c r="G514" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="515" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A515" t="s">
+        <v>434</v>
+      </c>
+      <c r="B515">
+        <v>2</v>
+      </c>
+      <c r="C515" t="s">
+        <v>187</v>
+      </c>
+      <c r="D515" t="s">
+        <v>208</v>
+      </c>
+      <c r="E515" t="s">
+        <v>239</v>
+      </c>
+      <c r="F515" t="s">
+        <v>196</v>
+      </c>
+      <c r="G515" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="516" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A516" t="s">
+        <v>434</v>
+      </c>
+      <c r="B516">
+        <v>2</v>
+      </c>
+      <c r="C516" t="s">
+        <v>191</v>
+      </c>
+      <c r="D516" t="s">
+        <v>208</v>
+      </c>
+      <c r="E516" t="s">
+        <v>239</v>
+      </c>
+      <c r="F516" t="s">
+        <v>196</v>
+      </c>
+      <c r="G516" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="517" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A517" t="s">
+        <v>453</v>
+      </c>
+      <c r="B517">
+        <v>2</v>
+      </c>
+      <c r="C517" t="s">
+        <v>187</v>
+      </c>
+      <c r="D517" t="s">
+        <v>208</v>
+      </c>
+      <c r="E517" t="s">
+        <v>193</v>
+      </c>
+      <c r="F517" t="s">
+        <v>216</v>
+      </c>
+      <c r="G517" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="518" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A518" t="s">
+        <v>455</v>
+      </c>
+      <c r="B518">
+        <v>2</v>
+      </c>
+      <c r="C518" t="s">
+        <v>187</v>
+      </c>
+      <c r="D518" t="s">
+        <v>180</v>
+      </c>
+      <c r="E518" t="s">
+        <v>186</v>
+      </c>
+      <c r="F518" t="s">
+        <v>196</v>
+      </c>
+      <c r="G518" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="519" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A519" t="s">
+        <v>457</v>
+      </c>
+      <c r="B519">
+        <v>2</v>
+      </c>
+      <c r="C519" t="s">
+        <v>184</v>
+      </c>
+      <c r="D519" t="s">
+        <v>188</v>
+      </c>
+      <c r="E519" t="s">
+        <v>234</v>
+      </c>
+      <c r="F519" t="s">
+        <v>196</v>
+      </c>
+      <c r="G519" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="520" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A520" t="s">
+        <v>451</v>
+      </c>
+      <c r="B520">
+        <v>3</v>
+      </c>
+      <c r="C520" t="s">
+        <v>179</v>
+      </c>
+      <c r="D520" t="s">
+        <v>221</v>
+      </c>
+      <c r="E520" t="s">
+        <v>201</v>
+      </c>
+      <c r="F520" t="s">
+        <v>182</v>
+      </c>
+      <c r="G520" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="521" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A521" t="s">
+        <v>434</v>
+      </c>
+      <c r="B521">
+        <v>3</v>
+      </c>
+      <c r="C521" t="s">
+        <v>184</v>
+      </c>
+      <c r="D521" t="s">
+        <v>185</v>
+      </c>
+      <c r="E521" t="s">
+        <v>186</v>
+      </c>
+      <c r="F521" t="s">
+        <v>196</v>
+      </c>
+      <c r="G521" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="522" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A522" t="s">
+        <v>434</v>
+      </c>
+      <c r="B522">
+        <v>3</v>
+      </c>
+      <c r="C522" t="s">
+        <v>179</v>
+      </c>
+      <c r="D522" t="s">
+        <v>185</v>
+      </c>
+      <c r="E522" t="s">
+        <v>186</v>
+      </c>
+      <c r="F522" t="s">
+        <v>196</v>
+      </c>
+      <c r="G522" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="523" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A523" t="s">
+        <v>457</v>
+      </c>
+      <c r="B523">
+        <v>3</v>
+      </c>
+      <c r="C523" t="s">
+        <v>187</v>
+      </c>
+      <c r="D523" t="s">
+        <v>208</v>
+      </c>
+      <c r="E523" t="s">
+        <v>209</v>
+      </c>
+      <c r="F523" t="s">
+        <v>196</v>
+      </c>
+      <c r="G523" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="524" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A524" t="s">
+        <v>460</v>
+      </c>
+      <c r="B524">
+        <v>3</v>
+      </c>
+      <c r="C524" t="s">
+        <v>191</v>
+      </c>
+      <c r="D524" t="s">
+        <v>208</v>
+      </c>
+      <c r="E524" t="s">
+        <v>193</v>
+      </c>
+      <c r="F524" t="s">
+        <v>196</v>
+      </c>
+      <c r="G524" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="525" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A525" t="s">
+        <v>451</v>
+      </c>
+      <c r="B525">
+        <v>4</v>
+      </c>
+      <c r="C525" t="s">
+        <v>187</v>
+      </c>
+      <c r="D525" t="s">
+        <v>208</v>
+      </c>
+      <c r="E525" t="s">
+        <v>209</v>
+      </c>
+      <c r="F525" t="s">
+        <v>182</v>
+      </c>
+      <c r="G525" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="526" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A526" t="s">
+        <v>434</v>
+      </c>
+      <c r="B526">
+        <v>4</v>
+      </c>
+      <c r="C526" t="s">
+        <v>187</v>
+      </c>
+      <c r="D526" t="s">
+        <v>188</v>
+      </c>
+      <c r="E526" t="s">
+        <v>189</v>
+      </c>
+      <c r="F526" t="s">
+        <v>182</v>
+      </c>
+      <c r="G526" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="527" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A527" t="s">
+        <v>434</v>
+      </c>
+      <c r="B527">
+        <v>4</v>
+      </c>
+      <c r="C527" t="s">
+        <v>191</v>
+      </c>
+      <c r="D527" t="s">
+        <v>188</v>
+      </c>
+      <c r="E527" t="s">
+        <v>189</v>
+      </c>
+      <c r="F527" t="s">
+        <v>182</v>
+      </c>
+      <c r="G527" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="528" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A528" t="s">
+        <v>451</v>
+      </c>
+      <c r="B528">
+        <v>5</v>
+      </c>
+      <c r="C528" t="s">
+        <v>187</v>
+      </c>
+      <c r="D528" t="s">
+        <v>185</v>
+      </c>
+      <c r="E528" t="s">
+        <v>206</v>
+      </c>
+      <c r="F528" t="s">
+        <v>216</v>
+      </c>
+      <c r="G528" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="529" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A529" t="s">
+        <v>434</v>
+      </c>
+      <c r="B529">
+        <v>5</v>
+      </c>
+      <c r="C529" t="s">
+        <v>275</v>
+      </c>
+      <c r="D529" t="s">
+        <v>180</v>
+      </c>
+      <c r="E529" t="s">
+        <v>186</v>
+      </c>
+      <c r="F529" t="s">
+        <v>247</v>
+      </c>
+      <c r="G529" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="530" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A530" t="s">
+        <v>451</v>
+      </c>
+      <c r="B530">
+        <v>6</v>
+      </c>
+      <c r="C530" t="s">
+        <v>187</v>
+      </c>
+      <c r="D530" t="s">
+        <v>221</v>
+      </c>
+      <c r="E530" t="s">
+        <v>201</v>
+      </c>
+      <c r="F530" t="s">
+        <v>216</v>
+      </c>
+      <c r="G530" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="531" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A531" t="s">
+        <v>434</v>
+      </c>
+      <c r="B531">
+        <v>6</v>
+      </c>
+      <c r="C531" t="s">
+        <v>187</v>
+      </c>
+      <c r="D531" t="s">
+        <v>192</v>
+      </c>
+      <c r="E531" t="s">
+        <v>193</v>
+      </c>
+      <c r="F531" t="s">
+        <v>196</v>
+      </c>
+      <c r="G531" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="532" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A532" t="s">
+        <v>434</v>
+      </c>
+      <c r="B532">
+        <v>6</v>
+      </c>
+      <c r="C532" t="s">
+        <v>191</v>
+      </c>
+      <c r="D532" t="s">
+        <v>192</v>
+      </c>
+      <c r="E532" t="s">
+        <v>193</v>
+      </c>
+      <c r="F532" t="s">
+        <v>196</v>
+      </c>
+      <c r="G532" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="533" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A533" t="s">
+        <v>451</v>
+      </c>
+      <c r="B533">
+        <v>7</v>
+      </c>
+      <c r="C533" t="s">
+        <v>187</v>
+      </c>
+      <c r="D533" t="s">
+        <v>221</v>
+      </c>
+      <c r="E533" t="s">
+        <v>201</v>
+      </c>
+      <c r="F533" t="s">
+        <v>182</v>
+      </c>
+      <c r="G533" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="534" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A534" t="s">
+        <v>434</v>
+      </c>
+      <c r="B534">
+        <v>7</v>
+      </c>
+      <c r="C534" t="s">
+        <v>184</v>
+      </c>
+      <c r="D534" t="s">
+        <v>188</v>
+      </c>
+      <c r="E534" t="s">
+        <v>189</v>
+      </c>
+      <c r="F534" t="s">
+        <v>196</v>
+      </c>
+      <c r="G534" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="535" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A535" t="s">
+        <v>434</v>
+      </c>
+      <c r="B535">
+        <v>7</v>
+      </c>
+      <c r="C535" t="s">
+        <v>179</v>
+      </c>
+      <c r="D535" t="s">
+        <v>188</v>
+      </c>
+      <c r="E535" t="s">
+        <v>189</v>
+      </c>
+      <c r="F535" t="s">
+        <v>196</v>
+      </c>
+      <c r="G535" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="536" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A536" t="s">
+        <v>451</v>
+      </c>
+      <c r="B536">
+        <v>8</v>
+      </c>
+      <c r="C536" t="s">
+        <v>204</v>
+      </c>
+      <c r="D536" t="s">
+        <v>221</v>
+      </c>
+      <c r="E536" t="s">
+        <v>201</v>
+      </c>
+      <c r="F536" t="s">
+        <v>182</v>
+      </c>
+      <c r="G536" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="537" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A537" t="s">
+        <v>434</v>
+      </c>
+      <c r="B537">
+        <v>8</v>
+      </c>
+      <c r="C537" t="s">
+        <v>184</v>
+      </c>
+      <c r="D537" t="s">
+        <v>188</v>
+      </c>
+      <c r="E537" t="s">
+        <v>189</v>
+      </c>
+      <c r="F537" t="s">
+        <v>289</v>
+      </c>
+      <c r="G537" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="538" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A538" t="s">
+        <v>434</v>
+      </c>
+      <c r="B538">
+        <v>8</v>
+      </c>
+      <c r="C538" t="s">
+        <v>179</v>
+      </c>
+      <c r="D538" t="s">
+        <v>188</v>
+      </c>
+      <c r="E538" t="s">
+        <v>189</v>
+      </c>
+      <c r="F538" t="s">
+        <v>289</v>
+      </c>
+      <c r="G538" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="539" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A539" t="s">
+        <v>451</v>
+      </c>
+      <c r="B539">
+        <v>9</v>
+      </c>
+      <c r="C539" t="s">
+        <v>179</v>
+      </c>
+      <c r="D539" t="s">
+        <v>185</v>
+      </c>
+      <c r="E539" t="s">
+        <v>206</v>
+      </c>
+      <c r="F539" t="s">
+        <v>216</v>
+      </c>
+      <c r="G539" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="540" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A540" t="s">
+        <v>434</v>
+      </c>
+      <c r="B540">
+        <v>9</v>
+      </c>
+      <c r="C540" t="s">
+        <v>275</v>
+      </c>
+      <c r="D540" t="s">
+        <v>180</v>
+      </c>
+      <c r="E540" t="s">
+        <v>186</v>
+      </c>
+      <c r="F540" t="s">
+        <v>247</v>
+      </c>
+      <c r="G540" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="541" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A541" t="s">
+        <v>451</v>
+      </c>
+      <c r="B541">
+        <v>10</v>
+      </c>
+      <c r="C541" t="s">
+        <v>179</v>
+      </c>
+      <c r="D541" t="s">
+        <v>208</v>
+      </c>
+      <c r="E541" t="s">
+        <v>209</v>
+      </c>
+      <c r="F541" t="s">
+        <v>182</v>
+      </c>
+      <c r="G541" t="s">
+        <v>215</v>
+      </c>
+      <c r="K541" s="11"/>
+    </row>
+    <row r="542" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A542" t="s">
+        <v>434</v>
+      </c>
+      <c r="B542">
+        <v>10</v>
+      </c>
+      <c r="C542" t="s">
+        <v>187</v>
+      </c>
+      <c r="D542" t="s">
+        <v>185</v>
+      </c>
+      <c r="E542" t="s">
+        <v>186</v>
+      </c>
+      <c r="F542" t="s">
+        <v>196</v>
+      </c>
+      <c r="G542" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="543" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A543" t="s">
+        <v>434</v>
+      </c>
+      <c r="B543">
+        <v>10</v>
+      </c>
+      <c r="C543" t="s">
+        <v>191</v>
+      </c>
+      <c r="D543" t="s">
+        <v>185</v>
+      </c>
+      <c r="E543" t="s">
+        <v>186</v>
+      </c>
+      <c r="F543" t="s">
+        <v>196</v>
+      </c>
+      <c r="G543" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="544" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A544" t="s">
+        <v>451</v>
+      </c>
+      <c r="B544">
+        <v>11</v>
+      </c>
+      <c r="C544" t="s">
+        <v>191</v>
+      </c>
+      <c r="D544" t="s">
+        <v>185</v>
+      </c>
+      <c r="E544" t="s">
+        <v>206</v>
+      </c>
+      <c r="F544" t="s">
+        <v>182</v>
+      </c>
+      <c r="G544" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="545" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A545" t="s">
+        <v>463</v>
+      </c>
+      <c r="B545">
+        <v>1</v>
+      </c>
+      <c r="C545" t="s">
+        <v>204</v>
+      </c>
+      <c r="D545" t="s">
+        <v>180</v>
+      </c>
+      <c r="E545" t="s">
+        <v>186</v>
+      </c>
+      <c r="F545" t="s">
+        <v>196</v>
+      </c>
+      <c r="G545" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="546" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A546" t="s">
+        <v>466</v>
+      </c>
+      <c r="B546">
+        <v>1</v>
+      </c>
+      <c r="C546" t="s">
+        <v>179</v>
+      </c>
+      <c r="D546" t="s">
+        <v>188</v>
+      </c>
+      <c r="E546" t="s">
+        <v>234</v>
+      </c>
+      <c r="F546" t="s">
+        <v>196</v>
+      </c>
+      <c r="G546" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="547" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A547" t="s">
+        <v>472</v>
+      </c>
+      <c r="B547">
+        <v>1</v>
+      </c>
+      <c r="C547" t="s">
+        <v>187</v>
+      </c>
+      <c r="D547" t="s">
+        <v>188</v>
+      </c>
+      <c r="E547" t="s">
+        <v>234</v>
+      </c>
+      <c r="F547" t="s">
+        <v>196</v>
+      </c>
+      <c r="G547" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="548" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A548" t="s">
+        <v>474</v>
+      </c>
+      <c r="B548">
+        <v>1</v>
+      </c>
+      <c r="C548" t="s">
+        <v>184</v>
+      </c>
+      <c r="D548" t="s">
+        <v>180</v>
+      </c>
+      <c r="E548" t="s">
+        <v>186</v>
+      </c>
+      <c r="F548" t="s">
+        <v>196</v>
+      </c>
+      <c r="G548" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="549" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A549" t="s">
+        <v>471</v>
+      </c>
+      <c r="B549">
+        <v>1</v>
+      </c>
+      <c r="C549" t="s">
+        <v>179</v>
+      </c>
+      <c r="D549" t="s">
+        <v>208</v>
+      </c>
+      <c r="E549" t="s">
+        <v>193</v>
+      </c>
+      <c r="F549" t="s">
+        <v>196</v>
+      </c>
+      <c r="G549" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="550" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A550" t="s">
+        <v>463</v>
+      </c>
+      <c r="B550">
+        <v>2</v>
+      </c>
+      <c r="C550" t="s">
+        <v>179</v>
+      </c>
+      <c r="D550" t="s">
+        <v>208</v>
+      </c>
+      <c r="E550" t="s">
+        <v>193</v>
+      </c>
+      <c r="F550" t="s">
+        <v>196</v>
+      </c>
+      <c r="G550" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="551" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A551" t="s">
+        <v>466</v>
+      </c>
+      <c r="B551">
+        <v>2</v>
+      </c>
+      <c r="C551" t="s">
+        <v>184</v>
+      </c>
+      <c r="D551" t="s">
+        <v>188</v>
+      </c>
+      <c r="E551" t="s">
+        <v>234</v>
+      </c>
+      <c r="F551" t="s">
+        <v>196</v>
+      </c>
+      <c r="G551" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="552" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A552" t="s">
+        <v>469</v>
+      </c>
+      <c r="B552">
+        <v>2</v>
+      </c>
+      <c r="C552" t="s">
+        <v>187</v>
+      </c>
+      <c r="D552" t="s">
+        <v>208</v>
+      </c>
+      <c r="E552" t="s">
+        <v>209</v>
+      </c>
+      <c r="F552" t="s">
+        <v>196</v>
+      </c>
+      <c r="G552" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="553" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A553" t="s">
+        <v>472</v>
+      </c>
+      <c r="B553">
+        <v>2</v>
+      </c>
+      <c r="C553" t="s">
+        <v>191</v>
+      </c>
+      <c r="D553" t="s">
+        <v>180</v>
+      </c>
+      <c r="E553" t="s">
+        <v>212</v>
+      </c>
+      <c r="F553" t="s">
+        <v>196</v>
+      </c>
+      <c r="G553" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="554" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A554" t="s">
+        <v>474</v>
+      </c>
+      <c r="B554">
+        <v>2</v>
+      </c>
+      <c r="C554" t="s">
+        <v>191</v>
+      </c>
+      <c r="D554" t="s">
+        <v>208</v>
+      </c>
+      <c r="E554" t="s">
+        <v>193</v>
+      </c>
+      <c r="F554" t="s">
+        <v>196</v>
+      </c>
+      <c r="G554" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="555" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A555" t="s">
+        <v>471</v>
+      </c>
+      <c r="B555">
+        <v>2</v>
+      </c>
+      <c r="C555" t="s">
+        <v>204</v>
+      </c>
+      <c r="D555" t="s">
+        <v>180</v>
+      </c>
+      <c r="E555" t="s">
+        <v>186</v>
+      </c>
+      <c r="F555" t="s">
+        <v>196</v>
+      </c>
+      <c r="G555" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="556" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A556" t="s">
+        <v>463</v>
+      </c>
+      <c r="B556">
+        <v>3</v>
+      </c>
+      <c r="C556" t="s">
+        <v>179</v>
+      </c>
+      <c r="D556" t="s">
+        <v>180</v>
+      </c>
+      <c r="E556" t="s">
+        <v>186</v>
+      </c>
+      <c r="F556" t="s">
+        <v>196</v>
+      </c>
+      <c r="G556" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="557" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A557" t="s">
+        <v>463</v>
+      </c>
+      <c r="B557">
+        <v>4</v>
+      </c>
+      <c r="C557" t="s">
+        <v>179</v>
+      </c>
+      <c r="D557" t="s">
+        <v>188</v>
+      </c>
+      <c r="E557" t="s">
+        <v>201</v>
+      </c>
+      <c r="F557" t="s">
+        <v>196</v>
+      </c>
+      <c r="G557" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="558" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A558" t="s">
+        <v>463</v>
+      </c>
+      <c r="B558">
+        <v>5</v>
+      </c>
+      <c r="C558" t="s">
+        <v>187</v>
+      </c>
+      <c r="D558" t="s">
+        <v>180</v>
+      </c>
+      <c r="E558" t="s">
+        <v>186</v>
+      </c>
+      <c r="F558" t="s">
+        <v>196</v>
+      </c>
+      <c r="G558" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="559" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A559" t="s">
+        <v>463</v>
+      </c>
+      <c r="B559">
+        <v>6</v>
+      </c>
+      <c r="C559" t="s">
+        <v>187</v>
+      </c>
+      <c r="D559" t="s">
+        <v>188</v>
+      </c>
+      <c r="E559" t="s">
+        <v>201</v>
+      </c>
+      <c r="F559" t="s">
+        <v>196</v>
+      </c>
+      <c r="G559" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="560" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A560" t="s">
+        <v>463</v>
+      </c>
+      <c r="B560">
+        <v>7</v>
+      </c>
+      <c r="C560" t="s">
+        <v>191</v>
+      </c>
+      <c r="D560" t="s">
+        <v>180</v>
+      </c>
+      <c r="E560" t="s">
+        <v>186</v>
+      </c>
+      <c r="F560" t="s">
+        <v>196</v>
+      </c>
+      <c r="G560" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="561" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A561" t="s">
+        <v>463</v>
+      </c>
+      <c r="B561">
+        <v>8</v>
+      </c>
+      <c r="C561" t="s">
+        <v>184</v>
+      </c>
+      <c r="D561" t="s">
+        <v>208</v>
+      </c>
+      <c r="E561" t="s">
+        <v>193</v>
+      </c>
+      <c r="F561" t="s">
+        <v>196</v>
+      </c>
+      <c r="G561" t="s">
+        <v>510</v>
       </c>
     </row>
   </sheetData>

</xml_diff>